<commit_message>
correction arrow et glass bottle on a mis les ingredients
</commit_message>
<xml_diff>
--- a/Musee_Infinis_clean_with_totals.xlsx
+++ b/Musee_Infinis_clean_with_totals.xlsx
@@ -481,7 +481,7 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Total ? farm</t>
+          <t>Total à farm</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
@@ -511,7 +511,7 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>33902</v>
+        <v>38762</v>
       </c>
       <c r="I2" t="n">
         <v>1728</v>
@@ -565,7 +565,7 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>6192</v>
       </c>
       <c r="I4" t="n">
         <v>1728</v>
@@ -916,7 +916,7 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>0</v>
+        <v>6192</v>
       </c>
       <c r="I17" t="n">
         <v>1728</v>
@@ -1267,7 +1267,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>0</v>
+        <v>6192</v>
       </c>
       <c r="I30" t="n">
         <v>1728</v>
@@ -1618,7 +1618,7 @@
         </is>
       </c>
       <c r="H43" t="n">
-        <v>0</v>
+        <v>6192</v>
       </c>
       <c r="I43" t="n">
         <v>1728</v>
@@ -1969,7 +1969,7 @@
         </is>
       </c>
       <c r="H56" t="n">
-        <v>0</v>
+        <v>6192</v>
       </c>
       <c r="I56" t="n">
         <v>1728</v>
@@ -2320,7 +2320,7 @@
         </is>
       </c>
       <c r="H69" t="n">
-        <v>0</v>
+        <v>6192</v>
       </c>
       <c r="I69" t="n">
         <v>1728</v>
@@ -2671,7 +2671,7 @@
         </is>
       </c>
       <c r="H82" t="n">
-        <v>0</v>
+        <v>6192</v>
       </c>
       <c r="I82" t="n">
         <v>1728</v>
@@ -3022,7 +3022,7 @@
         </is>
       </c>
       <c r="H95" t="n">
-        <v>0</v>
+        <v>6192</v>
       </c>
       <c r="I95" t="n">
         <v>1728</v>
@@ -3373,7 +3373,7 @@
         </is>
       </c>
       <c r="H108" t="n">
-        <v>0</v>
+        <v>6192</v>
       </c>
       <c r="I108" t="n">
         <v>1728</v>
@@ -3700,7 +3700,7 @@
         </is>
       </c>
       <c r="H120" t="n">
-        <v>0</v>
+        <v>3888</v>
       </c>
       <c r="I120" t="n">
         <v>1728</v>
@@ -4105,7 +4105,7 @@
         </is>
       </c>
       <c r="H135" t="n">
-        <v>0</v>
+        <v>6192</v>
       </c>
       <c r="I135" t="n">
         <v>1728</v>
@@ -4456,7 +4456,7 @@
         </is>
       </c>
       <c r="H148" t="n">
-        <v>0</v>
+        <v>6192</v>
       </c>
       <c r="I148" t="n">
         <v>1728</v>
@@ -4753,7 +4753,7 @@
         </is>
       </c>
       <c r="H159" t="n">
-        <v>0</v>
+        <v>46368</v>
       </c>
       <c r="I159" t="n">
         <v>1728</v>
@@ -4891,7 +4891,7 @@
         </is>
       </c>
       <c r="H164" t="n">
-        <v>162972</v>
+        <v>115776</v>
       </c>
       <c r="I164" t="n">
         <v>1728</v>
@@ -5119,7 +5119,7 @@
         </is>
       </c>
       <c r="H172" t="n">
-        <v>0</v>
+        <v>7992</v>
       </c>
       <c r="I172" t="n">
         <v>1728</v>
@@ -5200,7 +5200,7 @@
         </is>
       </c>
       <c r="H175" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I175" t="n">
         <v>1728</v>
@@ -6010,7 +6010,7 @@
         </is>
       </c>
       <c r="H205" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I205" t="n">
         <v>1728</v>
@@ -6037,7 +6037,7 @@
         </is>
       </c>
       <c r="H206" t="n">
-        <v>0</v>
+        <v>31104</v>
       </c>
       <c r="I206" t="n">
         <v>1728</v>
@@ -6307,7 +6307,7 @@
         </is>
       </c>
       <c r="H216" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I216" t="n">
         <v>1728</v>
@@ -6442,7 +6442,7 @@
         </is>
       </c>
       <c r="H221" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I221" t="n">
         <v>1728</v>
@@ -6550,7 +6550,7 @@
         </is>
       </c>
       <c r="H225" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I225" t="n">
         <v>1728</v>
@@ -6577,7 +6577,7 @@
         </is>
       </c>
       <c r="H226" t="n">
-        <v>0</v>
+        <v>24192</v>
       </c>
       <c r="I226" t="n">
         <v>1728</v>
@@ -7471,7 +7471,7 @@
         </is>
       </c>
       <c r="H259" t="n">
-        <v>0</v>
+        <v>5184</v>
       </c>
       <c r="I259" t="n">
         <v>1728</v>
@@ -7741,7 +7741,7 @@
         </is>
       </c>
       <c r="H269" t="n">
-        <v>0</v>
+        <v>5184</v>
       </c>
       <c r="I269" t="n">
         <v>1728</v>
@@ -8365,7 +8365,7 @@
         </is>
       </c>
       <c r="H292" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I292" t="n">
         <v>1728</v>
@@ -8527,7 +8527,7 @@
         </is>
       </c>
       <c r="H298" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I298" t="n">
         <v>1728</v>
@@ -8581,7 +8581,7 @@
         </is>
       </c>
       <c r="H300" t="n">
-        <v>28512</v>
+        <v>75708</v>
       </c>
       <c r="I300" t="n">
         <v>1728</v>
@@ -8608,7 +8608,7 @@
         </is>
       </c>
       <c r="H301" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I301" t="n">
         <v>1728</v>
@@ -8932,7 +8932,7 @@
         </is>
       </c>
       <c r="H313" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I313" t="n">
         <v>1728</v>
@@ -9202,7 +9202,7 @@
         </is>
       </c>
       <c r="H323" t="n">
-        <v>0</v>
+        <v>4320</v>
       </c>
       <c r="I323" t="n">
         <v>1728</v>
@@ -9823,7 +9823,7 @@
         </is>
       </c>
       <c r="H346" t="n">
-        <v>0</v>
+        <v>5184</v>
       </c>
       <c r="I346" t="n">
         <v>1728</v>
@@ -10228,7 +10228,7 @@
         </is>
       </c>
       <c r="H361" t="n">
-        <v>0</v>
+        <v>23328</v>
       </c>
       <c r="I361" t="n">
         <v>1728</v>
@@ -10390,7 +10390,7 @@
         </is>
       </c>
       <c r="H367" t="n">
-        <v>0</v>
+        <v>3456</v>
       </c>
       <c r="I367" t="n">
         <v>1728</v>
@@ -10417,7 +10417,7 @@
         </is>
       </c>
       <c r="H368" t="n">
-        <v>0</v>
+        <v>3456</v>
       </c>
       <c r="I368" t="n">
         <v>1728</v>
@@ -10444,7 +10444,7 @@
         </is>
       </c>
       <c r="H369" t="n">
-        <v>0</v>
+        <v>3456</v>
       </c>
       <c r="I369" t="n">
         <v>1728</v>
@@ -10498,7 +10498,7 @@
         </is>
       </c>
       <c r="H371" t="n">
-        <v>0</v>
+        <v>3456</v>
       </c>
       <c r="I371" t="n">
         <v>1728</v>
@@ -10525,7 +10525,7 @@
         </is>
       </c>
       <c r="H372" t="n">
-        <v>0</v>
+        <v>23328</v>
       </c>
       <c r="I372" t="n">
         <v>1728</v>
@@ -10687,7 +10687,7 @@
         </is>
       </c>
       <c r="H378" t="n">
-        <v>0</v>
+        <v>3456</v>
       </c>
       <c r="I378" t="n">
         <v>1728</v>
@@ -10714,7 +10714,7 @@
         </is>
       </c>
       <c r="H379" t="n">
-        <v>0</v>
+        <v>3456</v>
       </c>
       <c r="I379" t="n">
         <v>1728</v>
@@ -10741,7 +10741,7 @@
         </is>
       </c>
       <c r="H380" t="n">
-        <v>0</v>
+        <v>3456</v>
       </c>
       <c r="I380" t="n">
         <v>1728</v>
@@ -10795,7 +10795,7 @@
         </is>
       </c>
       <c r="H382" t="n">
-        <v>0</v>
+        <v>3456</v>
       </c>
       <c r="I382" t="n">
         <v>1728</v>
@@ -10822,7 +10822,7 @@
         </is>
       </c>
       <c r="H383" t="n">
-        <v>0</v>
+        <v>23328</v>
       </c>
       <c r="I383" t="n">
         <v>1728</v>
@@ -10984,7 +10984,7 @@
         </is>
       </c>
       <c r="H389" t="n">
-        <v>0</v>
+        <v>3456</v>
       </c>
       <c r="I389" t="n">
         <v>1728</v>
@@ -11011,7 +11011,7 @@
         </is>
       </c>
       <c r="H390" t="n">
-        <v>0</v>
+        <v>3456</v>
       </c>
       <c r="I390" t="n">
         <v>1728</v>
@@ -11038,7 +11038,7 @@
         </is>
       </c>
       <c r="H391" t="n">
-        <v>0</v>
+        <v>3456</v>
       </c>
       <c r="I391" t="n">
         <v>1728</v>
@@ -11092,7 +11092,7 @@
         </is>
       </c>
       <c r="H393" t="n">
-        <v>0</v>
+        <v>3456</v>
       </c>
       <c r="I393" t="n">
         <v>1728</v>
@@ -11119,7 +11119,7 @@
         </is>
       </c>
       <c r="H394" t="n">
-        <v>0</v>
+        <v>2592</v>
       </c>
       <c r="I394" t="n">
         <v>1728</v>
@@ -12388,7 +12388,7 @@
         </is>
       </c>
       <c r="H441" t="n">
-        <v>0</v>
+        <v>82080</v>
       </c>
       <c r="I441" t="n">
         <v>1728</v>
@@ -13171,7 +13171,7 @@
         </is>
       </c>
       <c r="H470" t="n">
-        <v>0</v>
+        <v>32832</v>
       </c>
       <c r="I470" t="n">
         <v>1728</v>
@@ -13630,7 +13630,7 @@
         </is>
       </c>
       <c r="H487" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I487" t="n">
         <v>1728</v>
@@ -13657,7 +13657,7 @@
         </is>
       </c>
       <c r="H488" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I488" t="n">
         <v>1728</v>
@@ -13684,7 +13684,7 @@
         </is>
       </c>
       <c r="H489" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I489" t="n">
         <v>1728</v>
@@ -13711,7 +13711,7 @@
         </is>
       </c>
       <c r="H490" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I490" t="n">
         <v>1728</v>
@@ -13738,7 +13738,7 @@
         </is>
       </c>
       <c r="H491" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I491" t="n">
         <v>1728</v>
@@ -13765,7 +13765,7 @@
         </is>
       </c>
       <c r="H492" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I492" t="n">
         <v>1728</v>
@@ -13792,7 +13792,7 @@
         </is>
       </c>
       <c r="H493" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I493" t="n">
         <v>1728</v>
@@ -13819,7 +13819,7 @@
         </is>
       </c>
       <c r="H494" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I494" t="n">
         <v>1728</v>
@@ -13846,7 +13846,7 @@
         </is>
       </c>
       <c r="H495" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I495" t="n">
         <v>1728</v>
@@ -13873,7 +13873,7 @@
         </is>
       </c>
       <c r="H496" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I496" t="n">
         <v>1728</v>
@@ -13900,7 +13900,7 @@
         </is>
       </c>
       <c r="H497" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I497" t="n">
         <v>1728</v>
@@ -13927,7 +13927,7 @@
         </is>
       </c>
       <c r="H498" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I498" t="n">
         <v>1728</v>
@@ -13954,7 +13954,7 @@
         </is>
       </c>
       <c r="H499" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I499" t="n">
         <v>1728</v>
@@ -13981,7 +13981,7 @@
         </is>
       </c>
       <c r="H500" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I500" t="n">
         <v>1728</v>
@@ -14008,7 +14008,7 @@
         </is>
       </c>
       <c r="H501" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I501" t="n">
         <v>1728</v>
@@ -14035,7 +14035,7 @@
         </is>
       </c>
       <c r="H502" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I502" t="n">
         <v>1728</v>
@@ -14494,7 +14494,7 @@
         </is>
       </c>
       <c r="H519" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I519" t="n">
         <v>1728</v>
@@ -14521,7 +14521,7 @@
         </is>
       </c>
       <c r="H520" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I520" t="n">
         <v>1728</v>
@@ -14548,7 +14548,7 @@
         </is>
       </c>
       <c r="H521" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I521" t="n">
         <v>1728</v>
@@ -14575,7 +14575,7 @@
         </is>
       </c>
       <c r="H522" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I522" t="n">
         <v>1728</v>
@@ -14602,7 +14602,7 @@
         </is>
       </c>
       <c r="H523" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I523" t="n">
         <v>1728</v>
@@ -14629,7 +14629,7 @@
         </is>
       </c>
       <c r="H524" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I524" t="n">
         <v>1728</v>
@@ -14656,7 +14656,7 @@
         </is>
       </c>
       <c r="H525" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I525" t="n">
         <v>1728</v>
@@ -14683,7 +14683,7 @@
         </is>
       </c>
       <c r="H526" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I526" t="n">
         <v>1728</v>
@@ -14710,7 +14710,7 @@
         </is>
       </c>
       <c r="H527" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I527" t="n">
         <v>1728</v>
@@ -14737,7 +14737,7 @@
         </is>
       </c>
       <c r="H528" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I528" t="n">
         <v>1728</v>
@@ -14764,7 +14764,7 @@
         </is>
       </c>
       <c r="H529" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I529" t="n">
         <v>1728</v>
@@ -14791,7 +14791,7 @@
         </is>
       </c>
       <c r="H530" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I530" t="n">
         <v>1728</v>
@@ -14818,7 +14818,7 @@
         </is>
       </c>
       <c r="H531" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I531" t="n">
         <v>1728</v>
@@ -14845,7 +14845,7 @@
         </is>
       </c>
       <c r="H532" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I532" t="n">
         <v>1728</v>
@@ -14872,7 +14872,7 @@
         </is>
       </c>
       <c r="H533" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I533" t="n">
         <v>1728</v>
@@ -14899,7 +14899,7 @@
         </is>
       </c>
       <c r="H534" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I534" t="n">
         <v>1728</v>
@@ -14929,7 +14929,7 @@
         </is>
       </c>
       <c r="H535" t="n">
-        <v>0</v>
+        <v>76302</v>
       </c>
       <c r="I535" t="n">
         <v>1728</v>
@@ -15904,7 +15904,7 @@
         </is>
       </c>
       <c r="H571" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I571" t="n">
         <v>27</v>
@@ -15931,7 +15931,7 @@
         </is>
       </c>
       <c r="H572" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I572" t="n">
         <v>27</v>
@@ -15958,7 +15958,7 @@
         </is>
       </c>
       <c r="H573" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I573" t="n">
         <v>27</v>
@@ -15985,7 +15985,7 @@
         </is>
       </c>
       <c r="H574" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I574" t="n">
         <v>27</v>
@@ -16012,7 +16012,7 @@
         </is>
       </c>
       <c r="H575" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I575" t="n">
         <v>27</v>
@@ -16039,7 +16039,7 @@
         </is>
       </c>
       <c r="H576" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I576" t="n">
         <v>27</v>
@@ -16066,7 +16066,7 @@
         </is>
       </c>
       <c r="H577" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I577" t="n">
         <v>27</v>
@@ -16093,7 +16093,7 @@
         </is>
       </c>
       <c r="H578" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I578" t="n">
         <v>27</v>
@@ -16120,7 +16120,7 @@
         </is>
       </c>
       <c r="H579" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I579" t="n">
         <v>27</v>
@@ -16147,7 +16147,7 @@
         </is>
       </c>
       <c r="H580" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I580" t="n">
         <v>27</v>
@@ -16174,7 +16174,7 @@
         </is>
       </c>
       <c r="H581" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I581" t="n">
         <v>27</v>
@@ -16201,7 +16201,7 @@
         </is>
       </c>
       <c r="H582" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I582" t="n">
         <v>27</v>
@@ -16228,7 +16228,7 @@
         </is>
       </c>
       <c r="H583" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I583" t="n">
         <v>27</v>
@@ -16255,7 +16255,7 @@
         </is>
       </c>
       <c r="H584" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I584" t="n">
         <v>27</v>
@@ -16282,7 +16282,7 @@
         </is>
       </c>
       <c r="H585" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I585" t="n">
         <v>27</v>
@@ -16309,7 +16309,7 @@
         </is>
       </c>
       <c r="H586" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I586" t="n">
         <v>27</v>
@@ -16417,7 +16417,7 @@
         </is>
       </c>
       <c r="H590" t="n">
-        <v>0</v>
+        <v>405</v>
       </c>
       <c r="I590" t="n">
         <v>27</v>
@@ -17662,7 +17662,7 @@
         </is>
       </c>
       <c r="H636" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I636" t="n">
         <v>1728</v>
@@ -17689,7 +17689,7 @@
         </is>
       </c>
       <c r="H637" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I637" t="n">
         <v>1728</v>
@@ -17716,7 +17716,7 @@
         </is>
       </c>
       <c r="H638" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I638" t="n">
         <v>1728</v>
@@ -17743,7 +17743,7 @@
         </is>
       </c>
       <c r="H639" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I639" t="n">
         <v>1728</v>
@@ -17773,7 +17773,7 @@
         </is>
       </c>
       <c r="H640" t="n">
-        <v>0</v>
+        <v>2592</v>
       </c>
       <c r="I640" t="n">
         <v>1728</v>
@@ -17827,7 +17827,7 @@
         </is>
       </c>
       <c r="H642" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I642" t="n">
         <v>1728</v>
@@ -17881,7 +17881,7 @@
         </is>
       </c>
       <c r="H644" t="n">
-        <v>0</v>
+        <v>12096</v>
       </c>
       <c r="I644" t="n">
         <v>1728</v>
@@ -17965,7 +17965,7 @@
         </is>
       </c>
       <c r="H647" t="n">
-        <v>63936</v>
+        <v>67608</v>
       </c>
       <c r="I647" t="n">
         <v>1728</v>
@@ -18019,7 +18019,7 @@
         </is>
       </c>
       <c r="H649" t="n">
-        <v>0</v>
+        <v>157248</v>
       </c>
       <c r="I649" t="n">
         <v>1728</v>
@@ -18154,7 +18154,7 @@
         </is>
       </c>
       <c r="H654" t="n">
-        <v>0</v>
+        <v>17568</v>
       </c>
       <c r="I654" t="n">
         <v>1728</v>
@@ -18208,7 +18208,7 @@
         </is>
       </c>
       <c r="H656" t="n">
-        <v>0</v>
+        <v>2880</v>
       </c>
       <c r="I656" t="n">
         <v>1728</v>
@@ -18262,7 +18262,7 @@
         </is>
       </c>
       <c r="H658" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I658" t="n">
         <v>1728</v>
@@ -18289,7 +18289,7 @@
         </is>
       </c>
       <c r="H659" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I659" t="n">
         <v>1728</v>
@@ -18343,7 +18343,7 @@
         </is>
       </c>
       <c r="H661" t="n">
-        <v>0</v>
+        <v>8640</v>
       </c>
       <c r="I661" t="n">
         <v>1728</v>
@@ -18424,7 +18424,7 @@
         </is>
       </c>
       <c r="H664" t="n">
-        <v>0</v>
+        <v>12096</v>
       </c>
       <c r="I664" t="n">
         <v>1728</v>
@@ -18451,7 +18451,7 @@
         </is>
       </c>
       <c r="H665" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I665" t="n">
         <v>1728</v>
@@ -18478,7 +18478,7 @@
         </is>
       </c>
       <c r="H666" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I666" t="n">
         <v>1728</v>
@@ -18505,7 +18505,7 @@
         </is>
       </c>
       <c r="H667" t="n">
-        <v>0</v>
+        <v>6048</v>
       </c>
       <c r="I667" t="n">
         <v>1728</v>
@@ -18532,7 +18532,7 @@
         </is>
       </c>
       <c r="H668" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I668" t="n">
         <v>1728</v>
@@ -18586,7 +18586,7 @@
         </is>
       </c>
       <c r="H670" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I670" t="n">
         <v>1728</v>
@@ -18613,7 +18613,7 @@
         </is>
       </c>
       <c r="H671" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I671" t="n">
         <v>1728</v>
@@ -18640,7 +18640,7 @@
         </is>
       </c>
       <c r="H672" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I672" t="n">
         <v>1728</v>
@@ -18667,7 +18667,7 @@
         </is>
       </c>
       <c r="H673" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I673" t="n">
         <v>1728</v>
@@ -18694,7 +18694,7 @@
         </is>
       </c>
       <c r="H674" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I674" t="n">
         <v>1728</v>
@@ -18721,7 +18721,7 @@
         </is>
       </c>
       <c r="H675" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I675" t="n">
         <v>1728</v>
@@ -18748,7 +18748,7 @@
         </is>
       </c>
       <c r="H676" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I676" t="n">
         <v>1728</v>
@@ -18775,7 +18775,7 @@
         </is>
       </c>
       <c r="H677" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I677" t="n">
         <v>1728</v>
@@ -18802,7 +18802,7 @@
         </is>
       </c>
       <c r="H678" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I678" t="n">
         <v>1728</v>
@@ -18829,7 +18829,7 @@
         </is>
       </c>
       <c r="H679" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I679" t="n">
         <v>1728</v>
@@ -18856,7 +18856,7 @@
         </is>
       </c>
       <c r="H680" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I680" t="n">
         <v>1728</v>
@@ -18883,7 +18883,7 @@
         </is>
       </c>
       <c r="H681" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I681" t="n">
         <v>1728</v>
@@ -18910,7 +18910,7 @@
         </is>
       </c>
       <c r="H682" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I682" t="n">
         <v>1728</v>
@@ -18937,7 +18937,7 @@
         </is>
       </c>
       <c r="H683" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I683" t="n">
         <v>1728</v>
@@ -18964,7 +18964,7 @@
         </is>
       </c>
       <c r="H684" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I684" t="n">
         <v>1728</v>
@@ -18991,7 +18991,7 @@
         </is>
       </c>
       <c r="H685" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I685" t="n">
         <v>1728</v>
@@ -19018,7 +19018,7 @@
         </is>
       </c>
       <c r="H686" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I686" t="n">
         <v>1728</v>
@@ -19045,7 +19045,7 @@
         </is>
       </c>
       <c r="H687" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I687" t="n">
         <v>1728</v>
@@ -19207,7 +19207,7 @@
         </is>
       </c>
       <c r="H693" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I693" t="n">
         <v>1728</v>
@@ -19234,7 +19234,7 @@
         </is>
       </c>
       <c r="H694" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I694" t="n">
         <v>1728</v>
@@ -19261,7 +19261,7 @@
         </is>
       </c>
       <c r="H695" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I695" t="n">
         <v>1728</v>
@@ -19288,7 +19288,7 @@
         </is>
       </c>
       <c r="H696" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I696" t="n">
         <v>1728</v>
@@ -19315,7 +19315,7 @@
         </is>
       </c>
       <c r="H697" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I697" t="n">
         <v>1728</v>
@@ -19342,7 +19342,7 @@
         </is>
       </c>
       <c r="H698" t="n">
-        <v>0</v>
+        <v>3456</v>
       </c>
       <c r="I698" t="n">
         <v>1728</v>
@@ -19396,7 +19396,7 @@
         </is>
       </c>
       <c r="H700" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I700" t="n">
         <v>1728</v>
@@ -19423,7 +19423,7 @@
         </is>
       </c>
       <c r="H701" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I701" t="n">
         <v>1728</v>
@@ -19450,7 +19450,7 @@
         </is>
       </c>
       <c r="H702" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I702" t="n">
         <v>1728</v>
@@ -19477,7 +19477,7 @@
         </is>
       </c>
       <c r="H703" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I703" t="n">
         <v>1728</v>
@@ -19504,7 +19504,7 @@
         </is>
       </c>
       <c r="H704" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I704" t="n">
         <v>1728</v>
@@ -19531,7 +19531,7 @@
         </is>
       </c>
       <c r="H705" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I705" t="n">
         <v>1728</v>
@@ -19558,7 +19558,7 @@
         </is>
       </c>
       <c r="H706" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I706" t="n">
         <v>1728</v>
@@ -19585,7 +19585,7 @@
         </is>
       </c>
       <c r="H707" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I707" t="n">
         <v>1728</v>
@@ -19612,7 +19612,7 @@
         </is>
       </c>
       <c r="H708" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I708" t="n">
         <v>1728</v>
@@ -19639,7 +19639,7 @@
         </is>
       </c>
       <c r="H709" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I709" t="n">
         <v>1728</v>
@@ -19666,7 +19666,7 @@
         </is>
       </c>
       <c r="H710" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I710" t="n">
         <v>1728</v>
@@ -19693,7 +19693,7 @@
         </is>
       </c>
       <c r="H711" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I711" t="n">
         <v>1728</v>
@@ -19720,7 +19720,7 @@
         </is>
       </c>
       <c r="H712" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I712" t="n">
         <v>1728</v>
@@ -19747,7 +19747,7 @@
         </is>
       </c>
       <c r="H713" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I713" t="n">
         <v>1728</v>
@@ -19801,7 +19801,7 @@
         </is>
       </c>
       <c r="H715" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I715" t="n">
         <v>1728</v>
@@ -19828,7 +19828,7 @@
         </is>
       </c>
       <c r="H716" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I716" t="n">
         <v>1728</v>
@@ -19855,7 +19855,7 @@
         </is>
       </c>
       <c r="H717" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I717" t="n">
         <v>1728</v>
@@ -19882,7 +19882,7 @@
         </is>
       </c>
       <c r="H718" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I718" t="n">
         <v>1728</v>
@@ -19909,7 +19909,7 @@
         </is>
       </c>
       <c r="H719" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I719" t="n">
         <v>1728</v>
@@ -19936,7 +19936,7 @@
         </is>
       </c>
       <c r="H720" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I720" t="n">
         <v>1728</v>
@@ -19963,7 +19963,7 @@
         </is>
       </c>
       <c r="H721" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I721" t="n">
         <v>1728</v>
@@ -19990,7 +19990,7 @@
         </is>
       </c>
       <c r="H722" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I722" t="n">
         <v>1728</v>
@@ -20017,7 +20017,7 @@
         </is>
       </c>
       <c r="H723" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I723" t="n">
         <v>1728</v>
@@ -20044,7 +20044,7 @@
         </is>
       </c>
       <c r="H724" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I724" t="n">
         <v>1728</v>
@@ -20071,7 +20071,7 @@
         </is>
       </c>
       <c r="H725" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I725" t="n">
         <v>1728</v>
@@ -20098,7 +20098,7 @@
         </is>
       </c>
       <c r="H726" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I726" t="n">
         <v>1728</v>
@@ -20125,7 +20125,7 @@
         </is>
       </c>
       <c r="H727" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I727" t="n">
         <v>1728</v>
@@ -20152,7 +20152,7 @@
         </is>
       </c>
       <c r="H728" t="n">
-        <v>0</v>
+        <v>3537</v>
       </c>
       <c r="I728" t="n">
         <v>1728</v>
@@ -20179,7 +20179,7 @@
         </is>
       </c>
       <c r="H729" t="n">
-        <v>0</v>
+        <v>1782</v>
       </c>
       <c r="I729" t="n">
         <v>1728</v>
@@ -20206,7 +20206,7 @@
         </is>
       </c>
       <c r="H730" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I730" t="n">
         <v>1728</v>
@@ -20233,7 +20233,7 @@
         </is>
       </c>
       <c r="H731" t="n">
-        <v>0</v>
+        <v>1755</v>
       </c>
       <c r="I731" t="n">
         <v>1728</v>
@@ -20260,7 +20260,7 @@
         </is>
       </c>
       <c r="H732" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I732" t="n">
         <v>1728</v>
@@ -20287,7 +20287,7 @@
         </is>
       </c>
       <c r="H733" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I733" t="n">
         <v>1728</v>
@@ -20314,7 +20314,7 @@
         </is>
       </c>
       <c r="H734" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I734" t="n">
         <v>1728</v>
@@ -20341,7 +20341,7 @@
         </is>
       </c>
       <c r="H735" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I735" t="n">
         <v>1728</v>
@@ -20368,7 +20368,7 @@
         </is>
       </c>
       <c r="H736" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I736" t="n">
         <v>1728</v>
@@ -20395,7 +20395,7 @@
         </is>
       </c>
       <c r="H737" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I737" t="n">
         <v>1728</v>
@@ -20422,7 +20422,7 @@
         </is>
       </c>
       <c r="H738" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I738" t="n">
         <v>1728</v>
@@ -20449,7 +20449,7 @@
         </is>
       </c>
       <c r="H739" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I739" t="n">
         <v>1728</v>
@@ -20476,7 +20476,7 @@
         </is>
       </c>
       <c r="H740" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I740" t="n">
         <v>1728</v>
@@ -20503,7 +20503,7 @@
         </is>
       </c>
       <c r="H741" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I741" t="n">
         <v>1728</v>
@@ -20530,7 +20530,7 @@
         </is>
       </c>
       <c r="H742" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I742" t="n">
         <v>1728</v>
@@ -20557,7 +20557,7 @@
         </is>
       </c>
       <c r="H743" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I743" t="n">
         <v>1728</v>
@@ -20584,7 +20584,7 @@
         </is>
       </c>
       <c r="H744" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I744" t="n">
         <v>1728</v>
@@ -20611,7 +20611,7 @@
         </is>
       </c>
       <c r="H745" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I745" t="n">
         <v>1728</v>
@@ -20638,7 +20638,7 @@
         </is>
       </c>
       <c r="H746" t="n">
-        <v>0</v>
+        <v>1755</v>
       </c>
       <c r="I746" t="n">
         <v>1728</v>
@@ -20665,7 +20665,7 @@
         </is>
       </c>
       <c r="H747" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I747" t="n">
         <v>1728</v>
@@ -20692,7 +20692,7 @@
         </is>
       </c>
       <c r="H748" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I748" t="n">
         <v>1728</v>
@@ -20719,7 +20719,7 @@
         </is>
       </c>
       <c r="H749" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I749" t="n">
         <v>1728</v>
@@ -20746,7 +20746,7 @@
         </is>
       </c>
       <c r="H750" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I750" t="n">
         <v>1728</v>
@@ -20773,7 +20773,7 @@
         </is>
       </c>
       <c r="H751" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I751" t="n">
         <v>1728</v>
@@ -20800,7 +20800,7 @@
         </is>
       </c>
       <c r="H752" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I752" t="n">
         <v>1728</v>
@@ -20827,7 +20827,7 @@
         </is>
       </c>
       <c r="H753" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I753" t="n">
         <v>1728</v>
@@ -20854,7 +20854,7 @@
         </is>
       </c>
       <c r="H754" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I754" t="n">
         <v>1728</v>
@@ -20881,7 +20881,7 @@
         </is>
       </c>
       <c r="H755" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I755" t="n">
         <v>1728</v>
@@ -20908,7 +20908,7 @@
         </is>
       </c>
       <c r="H756" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I756" t="n">
         <v>1728</v>
@@ -20935,7 +20935,7 @@
         </is>
       </c>
       <c r="H757" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I757" t="n">
         <v>1728</v>
@@ -20962,7 +20962,7 @@
         </is>
       </c>
       <c r="H758" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I758" t="n">
         <v>1728</v>
@@ -21046,7 +21046,7 @@
         </is>
       </c>
       <c r="H761" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I761" t="n">
         <v>1728</v>
@@ -21073,7 +21073,7 @@
         </is>
       </c>
       <c r="H762" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I762" t="n">
         <v>1728</v>
@@ -21100,7 +21100,7 @@
         </is>
       </c>
       <c r="H763" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I763" t="n">
         <v>1728</v>
@@ -21127,7 +21127,7 @@
         </is>
       </c>
       <c r="H764" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I764" t="n">
         <v>1728</v>
@@ -21154,7 +21154,7 @@
         </is>
       </c>
       <c r="H765" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I765" t="n">
         <v>1728</v>
@@ -21181,7 +21181,7 @@
         </is>
       </c>
       <c r="H766" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I766" t="n">
         <v>1728</v>
@@ -21208,7 +21208,7 @@
         </is>
       </c>
       <c r="H767" t="n">
-        <v>0</v>
+        <v>1755</v>
       </c>
       <c r="I767" t="n">
         <v>1728</v>
@@ -21235,7 +21235,7 @@
         </is>
       </c>
       <c r="H768" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I768" t="n">
         <v>1728</v>
@@ -21262,7 +21262,7 @@
         </is>
       </c>
       <c r="H769" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I769" t="n">
         <v>1728</v>
@@ -21289,7 +21289,7 @@
         </is>
       </c>
       <c r="H770" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I770" t="n">
         <v>1728</v>
@@ -21316,7 +21316,7 @@
         </is>
       </c>
       <c r="H771" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I771" t="n">
         <v>1728</v>
@@ -21343,7 +21343,7 @@
         </is>
       </c>
       <c r="H772" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I772" t="n">
         <v>1728</v>
@@ -21370,7 +21370,7 @@
         </is>
       </c>
       <c r="H773" t="n">
-        <v>0</v>
+        <v>16301</v>
       </c>
       <c r="I773" t="n">
         <v>1728</v>
@@ -21397,7 +21397,7 @@
         </is>
       </c>
       <c r="H774" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I774" t="n">
         <v>1728</v>
@@ -21424,7 +21424,7 @@
         </is>
       </c>
       <c r="H775" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I775" t="n">
         <v>1728</v>
@@ -21451,7 +21451,7 @@
         </is>
       </c>
       <c r="H776" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I776" t="n">
         <v>1728</v>
@@ -21478,7 +21478,7 @@
         </is>
       </c>
       <c r="H777" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I777" t="n">
         <v>1728</v>
@@ -21505,7 +21505,7 @@
         </is>
       </c>
       <c r="H778" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I778" t="n">
         <v>1728</v>
@@ -21532,7 +21532,7 @@
         </is>
       </c>
       <c r="H779" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I779" t="n">
         <v>1728</v>
@@ -21559,7 +21559,7 @@
         </is>
       </c>
       <c r="H780" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I780" t="n">
         <v>1728</v>
@@ -21586,7 +21586,7 @@
         </is>
       </c>
       <c r="H781" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I781" t="n">
         <v>1728</v>
@@ -21613,7 +21613,7 @@
         </is>
       </c>
       <c r="H782" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I782" t="n">
         <v>1728</v>
@@ -21640,7 +21640,7 @@
         </is>
       </c>
       <c r="H783" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I783" t="n">
         <v>1728</v>
@@ -21667,7 +21667,7 @@
         </is>
       </c>
       <c r="H784" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I784" t="n">
         <v>1728</v>
@@ -21724,7 +21724,7 @@
         </is>
       </c>
       <c r="H786" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I786" t="n">
         <v>1728</v>
@@ -21838,7 +21838,7 @@
         </is>
       </c>
       <c r="H790" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I790" t="n">
         <v>1728</v>
@@ -21865,7 +21865,7 @@
         </is>
       </c>
       <c r="H791" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I791" t="n">
         <v>1728</v>
@@ -21892,7 +21892,7 @@
         </is>
       </c>
       <c r="H792" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I792" t="n">
         <v>1728</v>
@@ -21919,7 +21919,7 @@
         </is>
       </c>
       <c r="H793" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I793" t="n">
         <v>1728</v>
@@ -21946,7 +21946,7 @@
         </is>
       </c>
       <c r="H794" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I794" t="n">
         <v>1728</v>
@@ -21973,7 +21973,7 @@
         </is>
       </c>
       <c r="H795" t="n">
-        <v>0</v>
+        <v>31104</v>
       </c>
       <c r="I795" t="n">
         <v>1728</v>
@@ -22000,7 +22000,7 @@
         </is>
       </c>
       <c r="H796" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I796" t="n">
         <v>1728</v>
@@ -22027,7 +22027,7 @@
         </is>
       </c>
       <c r="H797" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I797" t="n">
         <v>1728</v>
@@ -22054,7 +22054,7 @@
         </is>
       </c>
       <c r="H798" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I798" t="n">
         <v>1728</v>
@@ -22081,7 +22081,7 @@
         </is>
       </c>
       <c r="H799" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I799" t="n">
         <v>1728</v>
@@ -22108,7 +22108,7 @@
         </is>
       </c>
       <c r="H800" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I800" t="n">
         <v>1728</v>
@@ -22135,7 +22135,7 @@
         </is>
       </c>
       <c r="H801" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I801" t="n">
         <v>1728</v>
@@ -22162,7 +22162,7 @@
         </is>
       </c>
       <c r="H802" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I802" t="n">
         <v>1728</v>
@@ -22189,7 +22189,7 @@
         </is>
       </c>
       <c r="H803" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I803" t="n">
         <v>1728</v>
@@ -22216,7 +22216,7 @@
         </is>
       </c>
       <c r="H804" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I804" t="n">
         <v>1728</v>
@@ -22243,7 +22243,7 @@
         </is>
       </c>
       <c r="H805" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I805" t="n">
         <v>1728</v>
@@ -22270,7 +22270,7 @@
         </is>
       </c>
       <c r="H806" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I806" t="n">
         <v>1728</v>
@@ -22297,7 +22297,7 @@
         </is>
       </c>
       <c r="H807" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I807" t="n">
         <v>1728</v>
@@ -22324,7 +22324,7 @@
         </is>
       </c>
       <c r="H808" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I808" t="n">
         <v>1728</v>
@@ -22351,7 +22351,7 @@
         </is>
       </c>
       <c r="H809" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I809" t="n">
         <v>1728</v>
@@ -22378,7 +22378,7 @@
         </is>
       </c>
       <c r="H810" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I810" t="n">
         <v>1728</v>
@@ -22405,7 +22405,7 @@
         </is>
       </c>
       <c r="H811" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I811" t="n">
         <v>1728</v>
@@ -22432,7 +22432,7 @@
         </is>
       </c>
       <c r="H812" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I812" t="n">
         <v>1728</v>
@@ -22459,7 +22459,7 @@
         </is>
       </c>
       <c r="H813" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I813" t="n">
         <v>1728</v>
@@ -22486,7 +22486,7 @@
         </is>
       </c>
       <c r="H814" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I814" t="n">
         <v>1728</v>
@@ -22513,7 +22513,7 @@
         </is>
       </c>
       <c r="H815" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I815" t="n">
         <v>1728</v>
@@ -22540,7 +22540,7 @@
         </is>
       </c>
       <c r="H816" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I816" t="n">
         <v>1728</v>
@@ -22567,7 +22567,7 @@
         </is>
       </c>
       <c r="H817" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I817" t="n">
         <v>1728</v>
@@ -22594,7 +22594,7 @@
         </is>
       </c>
       <c r="H818" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I818" t="n">
         <v>1728</v>
@@ -22621,7 +22621,7 @@
         </is>
       </c>
       <c r="H819" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I819" t="n">
         <v>1728</v>
@@ -22648,7 +22648,7 @@
         </is>
       </c>
       <c r="H820" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I820" t="n">
         <v>1728</v>
@@ -22675,7 +22675,7 @@
         </is>
       </c>
       <c r="H821" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I821" t="n">
         <v>1728</v>
@@ -22702,7 +22702,7 @@
         </is>
       </c>
       <c r="H822" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I822" t="n">
         <v>1728</v>
@@ -22729,7 +22729,7 @@
         </is>
       </c>
       <c r="H823" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I823" t="n">
         <v>1728</v>
@@ -22756,7 +22756,7 @@
         </is>
       </c>
       <c r="H824" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I824" t="n">
         <v>1728</v>
@@ -22783,7 +22783,7 @@
         </is>
       </c>
       <c r="H825" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I825" t="n">
         <v>1728</v>
@@ -22810,7 +22810,7 @@
         </is>
       </c>
       <c r="H826" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I826" t="n">
         <v>1728</v>
@@ -22837,7 +22837,7 @@
         </is>
       </c>
       <c r="H827" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I827" t="n">
         <v>1728</v>
@@ -22864,7 +22864,7 @@
         </is>
       </c>
       <c r="H828" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I828" t="n">
         <v>1728</v>
@@ -22891,7 +22891,7 @@
         </is>
       </c>
       <c r="H829" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I829" t="n">
         <v>1728</v>
@@ -22918,7 +22918,7 @@
         </is>
       </c>
       <c r="H830" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I830" t="n">
         <v>1728</v>
@@ -22945,7 +22945,7 @@
         </is>
       </c>
       <c r="H831" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I831" t="n">
         <v>1728</v>
@@ -22972,7 +22972,7 @@
         </is>
       </c>
       <c r="H832" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I832" t="n">
         <v>1728</v>
@@ -23053,7 +23053,7 @@
         </is>
       </c>
       <c r="H835" t="n">
-        <v>0</v>
+        <v>3456</v>
       </c>
       <c r="I835" t="n">
         <v>1728</v>
@@ -23107,7 +23107,7 @@
         </is>
       </c>
       <c r="H837" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I837" t="n">
         <v>1728</v>
@@ -23188,7 +23188,7 @@
         </is>
       </c>
       <c r="H840" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I840" t="n">
         <v>1728</v>
@@ -23215,7 +23215,7 @@
         </is>
       </c>
       <c r="H841" t="n">
-        <v>0</v>
+        <v>3456</v>
       </c>
       <c r="I841" t="n">
         <v>1728</v>
@@ -23242,7 +23242,7 @@
         </is>
       </c>
       <c r="H842" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I842" t="n">
         <v>1728</v>
@@ -23269,7 +23269,7 @@
         </is>
       </c>
       <c r="H843" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I843" t="n">
         <v>1728</v>
@@ -23296,7 +23296,7 @@
         </is>
       </c>
       <c r="H844" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I844" t="n">
         <v>1728</v>
@@ -23323,7 +23323,7 @@
         </is>
       </c>
       <c r="H845" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I845" t="n">
         <v>1728</v>
@@ -23350,7 +23350,7 @@
         </is>
       </c>
       <c r="H846" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I846" t="n">
         <v>1728</v>
@@ -23377,7 +23377,7 @@
         </is>
       </c>
       <c r="H847" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I847" t="n">
         <v>1728</v>
@@ -23404,7 +23404,7 @@
         </is>
       </c>
       <c r="H848" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I848" t="n">
         <v>1728</v>
@@ -23431,7 +23431,7 @@
         </is>
       </c>
       <c r="H849" t="n">
-        <v>0</v>
+        <v>3456</v>
       </c>
       <c r="I849" t="n">
         <v>1728</v>
@@ -23458,7 +23458,7 @@
         </is>
       </c>
       <c r="H850" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I850" t="n">
         <v>1728</v>
@@ -23674,7 +23674,7 @@
         </is>
       </c>
       <c r="H858" t="n">
-        <v>0</v>
+        <v>3456</v>
       </c>
       <c r="I858" t="n">
         <v>1728</v>
@@ -23701,7 +23701,7 @@
         </is>
       </c>
       <c r="H859" t="n">
-        <v>0</v>
+        <v>3456</v>
       </c>
       <c r="I859" t="n">
         <v>1728</v>
@@ -23728,7 +23728,7 @@
         </is>
       </c>
       <c r="H860" t="n">
-        <v>0</v>
+        <v>3456</v>
       </c>
       <c r="I860" t="n">
         <v>1728</v>
@@ -24268,7 +24268,7 @@
         </is>
       </c>
       <c r="H880" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I880" t="n">
         <v>1728</v>
@@ -24295,7 +24295,7 @@
         </is>
       </c>
       <c r="H881" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I881" t="n">
         <v>1728</v>
@@ -24511,7 +24511,7 @@
         </is>
       </c>
       <c r="H889" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I889" t="n">
         <v>1728</v>
@@ -24703,7 +24703,7 @@
         </is>
       </c>
       <c r="H896" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I896" t="n">
         <v>1728</v>
@@ -24730,7 +24730,7 @@
         </is>
       </c>
       <c r="H897" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I897" t="n">
         <v>1728</v>
@@ -24784,7 +24784,7 @@
         </is>
       </c>
       <c r="H899" t="n">
-        <v>0</v>
+        <v>3456</v>
       </c>
       <c r="I899" t="n">
         <v>1728</v>
@@ -24811,7 +24811,7 @@
         </is>
       </c>
       <c r="H900" t="n">
-        <v>0</v>
+        <v>3456</v>
       </c>
       <c r="I900" t="n">
         <v>1728</v>
@@ -24838,7 +24838,7 @@
         </is>
       </c>
       <c r="H901" t="n">
-        <v>0</v>
+        <v>3456</v>
       </c>
       <c r="I901" t="n">
         <v>1728</v>
@@ -26242,7 +26242,7 @@
         </is>
       </c>
       <c r="H953" t="n">
-        <v>0</v>
+        <v>3456</v>
       </c>
       <c r="I953" t="n">
         <v>1728</v>
@@ -26269,7 +26269,7 @@
         </is>
       </c>
       <c r="H954" t="n">
-        <v>0</v>
+        <v>3456</v>
       </c>
       <c r="I954" t="n">
         <v>1728</v>
@@ -26296,7 +26296,7 @@
         </is>
       </c>
       <c r="H955" t="n">
-        <v>0</v>
+        <v>3456</v>
       </c>
       <c r="I955" t="n">
         <v>1728</v>
@@ -26512,7 +26512,7 @@
         </is>
       </c>
       <c r="H963" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I963" t="n">
         <v>1728</v>
@@ -26539,7 +26539,7 @@
         </is>
       </c>
       <c r="H964" t="n">
-        <v>0</v>
+        <v>1755</v>
       </c>
       <c r="I964" t="n">
         <v>1728</v>
@@ -26566,7 +26566,7 @@
         </is>
       </c>
       <c r="H965" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I965" t="n">
         <v>1728</v>
@@ -26593,7 +26593,7 @@
         </is>
       </c>
       <c r="H966" t="n">
-        <v>0</v>
+        <v>1755</v>
       </c>
       <c r="I966" t="n">
         <v>1728</v>
@@ -26620,7 +26620,7 @@
         </is>
       </c>
       <c r="H967" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I967" t="n">
         <v>1728</v>
@@ -26647,7 +26647,7 @@
         </is>
       </c>
       <c r="H968" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I968" t="n">
         <v>1728</v>
@@ -26674,7 +26674,7 @@
         </is>
       </c>
       <c r="H969" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I969" t="n">
         <v>1728</v>
@@ -26701,7 +26701,7 @@
         </is>
       </c>
       <c r="H970" t="n">
-        <v>0</v>
+        <v>3456</v>
       </c>
       <c r="I970" t="n">
         <v>1728</v>
@@ -26728,7 +26728,7 @@
         </is>
       </c>
       <c r="H971" t="n">
-        <v>0</v>
+        <v>3456</v>
       </c>
       <c r="I971" t="n">
         <v>1728</v>
@@ -26755,7 +26755,7 @@
         </is>
       </c>
       <c r="H972" t="n">
-        <v>0</v>
+        <v>3456</v>
       </c>
       <c r="I972" t="n">
         <v>1728</v>
@@ -26782,7 +26782,7 @@
         </is>
       </c>
       <c r="H973" t="n">
-        <v>0</v>
+        <v>3456</v>
       </c>
       <c r="I973" t="n">
         <v>1728</v>
@@ -26917,7 +26917,7 @@
         </is>
       </c>
       <c r="H978" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I978" t="n">
         <v>1728</v>
@@ -26944,7 +26944,7 @@
         </is>
       </c>
       <c r="H979" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I979" t="n">
         <v>1728</v>
@@ -26971,7 +26971,7 @@
         </is>
       </c>
       <c r="H980" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I980" t="n">
         <v>1728</v>
@@ -26998,7 +26998,7 @@
         </is>
       </c>
       <c r="H981" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I981" t="n">
         <v>1728</v>
@@ -27025,7 +27025,7 @@
         </is>
       </c>
       <c r="H982" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I982" t="n">
         <v>1728</v>
@@ -27052,7 +27052,7 @@
         </is>
       </c>
       <c r="H983" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I983" t="n">
         <v>1728</v>
@@ -27079,7 +27079,7 @@
         </is>
       </c>
       <c r="H984" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I984" t="n">
         <v>1728</v>
@@ -28399,7 +28399,7 @@
         </is>
       </c>
       <c r="H1032" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1032" t="n">
         <v>27</v>
@@ -28426,7 +28426,7 @@
         </is>
       </c>
       <c r="H1033" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1033" t="n">
         <v>27</v>
@@ -28453,7 +28453,7 @@
         </is>
       </c>
       <c r="H1034" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1034" t="n">
         <v>27</v>
@@ -28480,7 +28480,7 @@
         </is>
       </c>
       <c r="H1035" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1035" t="n">
         <v>27</v>
@@ -28534,7 +28534,7 @@
         </is>
       </c>
       <c r="H1037" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1037" t="n">
         <v>27</v>
@@ -28561,7 +28561,7 @@
         </is>
       </c>
       <c r="H1038" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1038" t="n">
         <v>27</v>
@@ -28588,7 +28588,7 @@
         </is>
       </c>
       <c r="H1039" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1039" t="n">
         <v>27</v>
@@ -28615,7 +28615,7 @@
         </is>
       </c>
       <c r="H1040" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1040" t="n">
         <v>27</v>
@@ -28642,7 +28642,7 @@
         </is>
       </c>
       <c r="H1041" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1041" t="n">
         <v>27</v>
@@ -28669,7 +28669,7 @@
         </is>
       </c>
       <c r="H1042" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1042" t="n">
         <v>27</v>
@@ -28696,7 +28696,7 @@
         </is>
       </c>
       <c r="H1043" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1043" t="n">
         <v>27</v>
@@ -28723,7 +28723,7 @@
         </is>
       </c>
       <c r="H1044" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1044" t="n">
         <v>27</v>
@@ -28750,7 +28750,7 @@
         </is>
       </c>
       <c r="H1045" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1045" t="n">
         <v>27</v>
@@ -28777,7 +28777,7 @@
         </is>
       </c>
       <c r="H1046" t="n">
-        <v>0</v>
+        <v>108</v>
       </c>
       <c r="I1046" t="n">
         <v>27</v>
@@ -28969,7 +28969,7 @@
         </is>
       </c>
       <c r="H1053" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I1053" t="n">
         <v>1728</v>
@@ -29050,7 +29050,7 @@
         </is>
       </c>
       <c r="H1056" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1056" t="n">
         <v>27</v>
@@ -29077,7 +29077,7 @@
         </is>
       </c>
       <c r="H1057" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1057" t="n">
         <v>27</v>
@@ -29104,7 +29104,7 @@
         </is>
       </c>
       <c r="H1058" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1058" t="n">
         <v>27</v>
@@ -29131,7 +29131,7 @@
         </is>
       </c>
       <c r="H1059" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1059" t="n">
         <v>27</v>
@@ -29158,7 +29158,7 @@
         </is>
       </c>
       <c r="H1060" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1060" t="n">
         <v>27</v>
@@ -29185,7 +29185,7 @@
         </is>
       </c>
       <c r="H1061" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1061" t="n">
         <v>27</v>
@@ -29212,7 +29212,7 @@
         </is>
       </c>
       <c r="H1062" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1062" t="n">
         <v>27</v>
@@ -29239,7 +29239,7 @@
         </is>
       </c>
       <c r="H1063" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1063" t="n">
         <v>27</v>
@@ -29266,7 +29266,7 @@
         </is>
       </c>
       <c r="H1064" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1064" t="n">
         <v>27</v>
@@ -29293,7 +29293,7 @@
         </is>
       </c>
       <c r="H1065" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1065" t="n">
         <v>27</v>
@@ -29320,7 +29320,7 @@
         </is>
       </c>
       <c r="H1066" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1066" t="n">
         <v>27</v>
@@ -29347,7 +29347,7 @@
         </is>
       </c>
       <c r="H1067" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1067" t="n">
         <v>27</v>
@@ -29374,7 +29374,7 @@
         </is>
       </c>
       <c r="H1068" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1068" t="n">
         <v>27</v>
@@ -29401,7 +29401,7 @@
         </is>
       </c>
       <c r="H1069" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1069" t="n">
         <v>27</v>
@@ -29428,7 +29428,7 @@
         </is>
       </c>
       <c r="H1070" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1070" t="n">
         <v>27</v>
@@ -29455,7 +29455,7 @@
         </is>
       </c>
       <c r="H1071" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1071" t="n">
         <v>27</v>
@@ -29725,7 +29725,7 @@
         </is>
       </c>
       <c r="H1081" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1081" t="n">
         <v>27</v>
@@ -29860,7 +29860,7 @@
         </is>
       </c>
       <c r="H1086" t="n">
-        <v>0</v>
+        <v>405</v>
       </c>
       <c r="I1086" t="n">
         <v>27</v>
@@ -30781,7 +30781,7 @@
         </is>
       </c>
       <c r="H1120" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1120" t="n">
         <v>27</v>
@@ -30976,7 +30976,7 @@
         </is>
       </c>
       <c r="H1127" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1127" t="n">
         <v>27</v>
@@ -31168,7 +31168,7 @@
         </is>
       </c>
       <c r="H1134" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1134" t="n">
         <v>27</v>
@@ -31195,7 +31195,7 @@
         </is>
       </c>
       <c r="H1135" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1135" t="n">
         <v>27</v>
@@ -31492,7 +31492,7 @@
         </is>
       </c>
       <c r="H1146" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1146" t="n">
         <v>27</v>
@@ -31519,7 +31519,7 @@
         </is>
       </c>
       <c r="H1147" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1147" t="n">
         <v>27</v>
@@ -31546,7 +31546,7 @@
         </is>
       </c>
       <c r="H1148" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1148" t="n">
         <v>27</v>
@@ -31573,7 +31573,7 @@
         </is>
       </c>
       <c r="H1149" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1149" t="n">
         <v>27</v>
@@ -31924,7 +31924,7 @@
         </is>
       </c>
       <c r="H1162" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1162" t="n">
         <v>27</v>
@@ -31951,7 +31951,7 @@
         </is>
       </c>
       <c r="H1163" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1163" t="n">
         <v>27</v>
@@ -31978,7 +31978,7 @@
         </is>
       </c>
       <c r="H1164" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1164" t="n">
         <v>27</v>
@@ -32005,7 +32005,7 @@
         </is>
       </c>
       <c r="H1165" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1165" t="n">
         <v>27</v>
@@ -32086,7 +32086,7 @@
         </is>
       </c>
       <c r="H1168" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1168" t="n">
         <v>27</v>
@@ -32113,7 +32113,7 @@
         </is>
       </c>
       <c r="H1169" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1169" t="n">
         <v>27</v>
@@ -32140,7 +32140,7 @@
         </is>
       </c>
       <c r="H1170" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1170" t="n">
         <v>27</v>
@@ -32167,7 +32167,7 @@
         </is>
       </c>
       <c r="H1171" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1171" t="n">
         <v>27</v>
@@ -32194,7 +32194,7 @@
         </is>
       </c>
       <c r="H1172" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1172" t="n">
         <v>27</v>
@@ -32248,7 +32248,7 @@
         </is>
       </c>
       <c r="H1174" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1174" t="n">
         <v>27</v>
@@ -32275,7 +32275,7 @@
         </is>
       </c>
       <c r="H1175" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1175" t="n">
         <v>27</v>
@@ -32302,7 +32302,7 @@
         </is>
       </c>
       <c r="H1176" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1176" t="n">
         <v>27</v>
@@ -32329,7 +32329,7 @@
         </is>
       </c>
       <c r="H1177" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1177" t="n">
         <v>27</v>
@@ -32356,7 +32356,7 @@
         </is>
       </c>
       <c r="H1178" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1178" t="n">
         <v>27</v>
@@ -32383,7 +32383,7 @@
         </is>
       </c>
       <c r="H1179" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1179" t="n">
         <v>27</v>
@@ -32410,7 +32410,7 @@
         </is>
       </c>
       <c r="H1180" t="n">
-        <v>0</v>
+        <v>10800</v>
       </c>
       <c r="I1180" t="n">
         <v>432</v>
@@ -32464,7 +32464,7 @@
         </is>
       </c>
       <c r="H1182" t="n">
-        <v>0</v>
+        <v>432</v>
       </c>
       <c r="I1182" t="n">
         <v>432</v>
@@ -32491,7 +32491,7 @@
         </is>
       </c>
       <c r="H1183" t="n">
-        <v>0</v>
+        <v>432</v>
       </c>
       <c r="I1183" t="n">
         <v>432</v>
@@ -32572,7 +32572,7 @@
         </is>
       </c>
       <c r="H1186" t="n">
-        <v>77760</v>
+        <v>0</v>
       </c>
       <c r="I1186" t="n">
         <v>1728</v>
@@ -32626,7 +32626,7 @@
         </is>
       </c>
       <c r="H1188" t="n">
-        <v>0</v>
+        <v>3456</v>
       </c>
       <c r="I1188" t="n">
         <v>1728</v>
@@ -32680,7 +32680,7 @@
         </is>
       </c>
       <c r="H1190" t="n">
-        <v>0</v>
+        <v>1755</v>
       </c>
       <c r="I1190" t="n">
         <v>1728</v>
@@ -32734,7 +32734,7 @@
         </is>
       </c>
       <c r="H1192" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I1192" t="n">
         <v>1728</v>
@@ -32764,7 +32764,7 @@
         </is>
       </c>
       <c r="H1193" t="n">
-        <v>0</v>
+        <v>3510</v>
       </c>
       <c r="I1193" t="n">
         <v>1728</v>
@@ -32821,7 +32821,7 @@
         </is>
       </c>
       <c r="H1195" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I1195" t="n">
         <v>1728</v>
@@ -32848,7 +32848,7 @@
         </is>
       </c>
       <c r="H1196" t="n">
-        <v>0</v>
+        <v>1755</v>
       </c>
       <c r="I1196" t="n">
         <v>1728</v>
@@ -32875,7 +32875,7 @@
         </is>
       </c>
       <c r="H1197" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I1197" t="n">
         <v>1728</v>
@@ -32905,7 +32905,7 @@
         </is>
       </c>
       <c r="H1198" t="n">
-        <v>0</v>
+        <v>1890</v>
       </c>
       <c r="I1198" t="n">
         <v>1728</v>
@@ -32932,7 +32932,7 @@
         </is>
       </c>
       <c r="H1199" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I1199" t="n">
         <v>1728</v>
@@ -32959,7 +32959,7 @@
         </is>
       </c>
       <c r="H1200" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I1200" t="n">
         <v>1728</v>
@@ -32986,7 +32986,7 @@
         </is>
       </c>
       <c r="H1201" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I1201" t="n">
         <v>1728</v>
@@ -33013,7 +33013,7 @@
         </is>
       </c>
       <c r="H1202" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I1202" t="n">
         <v>1728</v>
@@ -33040,7 +33040,7 @@
         </is>
       </c>
       <c r="H1203" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I1203" t="n">
         <v>1728</v>
@@ -33067,7 +33067,7 @@
         </is>
       </c>
       <c r="H1204" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I1204" t="n">
         <v>1728</v>
@@ -33094,7 +33094,7 @@
         </is>
       </c>
       <c r="H1205" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I1205" t="n">
         <v>1728</v>
@@ -33121,7 +33121,7 @@
         </is>
       </c>
       <c r="H1206" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I1206" t="n">
         <v>1728</v>
@@ -33148,7 +33148,7 @@
         </is>
       </c>
       <c r="H1207" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I1207" t="n">
         <v>1728</v>
@@ -33175,7 +33175,7 @@
         </is>
       </c>
       <c r="H1208" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I1208" t="n">
         <v>1728</v>
@@ -33202,7 +33202,7 @@
         </is>
       </c>
       <c r="H1209" t="n">
-        <v>0</v>
+        <v>1755</v>
       </c>
       <c r="I1209" t="n">
         <v>1728</v>
@@ -33229,7 +33229,7 @@
         </is>
       </c>
       <c r="H1210" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I1210" t="n">
         <v>1728</v>
@@ -33256,7 +33256,7 @@
         </is>
       </c>
       <c r="H1211" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I1211" t="n">
         <v>1728</v>
@@ -33283,7 +33283,7 @@
         </is>
       </c>
       <c r="H1212" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I1212" t="n">
         <v>1728</v>
@@ -33310,7 +33310,7 @@
         </is>
       </c>
       <c r="H1213" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I1213" t="n">
         <v>1728</v>
@@ -33337,7 +33337,7 @@
         </is>
       </c>
       <c r="H1214" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I1214" t="n">
         <v>1728</v>
@@ -33364,7 +33364,7 @@
         </is>
       </c>
       <c r="H1215" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I1215" t="n">
         <v>1728</v>
@@ -33499,7 +33499,7 @@
         </is>
       </c>
       <c r="H1220" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I1220" t="n">
         <v>1728</v>
@@ -33526,7 +33526,7 @@
         </is>
       </c>
       <c r="H1221" t="n">
-        <v>0</v>
+        <v>3456</v>
       </c>
       <c r="I1221" t="n">
         <v>1728</v>
@@ -33664,7 +33664,7 @@
         </is>
       </c>
       <c r="H1226" t="n">
-        <v>0</v>
+        <v>432</v>
       </c>
       <c r="I1226" t="n">
         <v>432</v>
@@ -34096,7 +34096,7 @@
         </is>
       </c>
       <c r="H1242" t="n">
-        <v>0</v>
+        <v>264897</v>
       </c>
       <c r="I1242" t="n">
         <v>1728</v>
@@ -34123,7 +34123,7 @@
         </is>
       </c>
       <c r="H1243" t="n">
-        <v>0</v>
+        <v>170150</v>
       </c>
       <c r="I1243" t="n">
         <v>1728</v>
@@ -34150,7 +34150,7 @@
         </is>
       </c>
       <c r="H1244" t="n">
-        <v>0</v>
+        <v>47436</v>
       </c>
       <c r="I1244" t="n">
         <v>1728</v>
@@ -34204,7 +34204,7 @@
         </is>
       </c>
       <c r="H1246" t="n">
-        <v>0</v>
+        <v>17280</v>
       </c>
       <c r="I1246" t="n">
         <v>1728</v>
@@ -34261,7 +34261,7 @@
         </is>
       </c>
       <c r="H1248" t="n">
-        <v>5859</v>
+        <v>25299</v>
       </c>
       <c r="I1248" t="n">
         <v>1728</v>
@@ -34345,7 +34345,7 @@
         </is>
       </c>
       <c r="H1251" t="n">
-        <v>2430</v>
+        <v>21870</v>
       </c>
       <c r="I1251" t="n">
         <v>1728</v>
@@ -34399,7 +34399,7 @@
         </is>
       </c>
       <c r="H1253" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I1253" t="n">
         <v>1728</v>
@@ -34453,7 +34453,7 @@
         </is>
       </c>
       <c r="H1255" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I1255" t="n">
         <v>1728</v>
@@ -34480,7 +34480,7 @@
         </is>
       </c>
       <c r="H1256" t="n">
-        <v>0</v>
+        <v>95774</v>
       </c>
       <c r="I1256" t="n">
         <v>1728</v>
@@ -34507,7 +34507,7 @@
         </is>
       </c>
       <c r="H1257" t="n">
-        <v>0</v>
+        <v>3456</v>
       </c>
       <c r="I1257" t="n">
         <v>1728</v>
@@ -34534,7 +34534,7 @@
         </is>
       </c>
       <c r="H1258" t="n">
-        <v>0</v>
+        <v>1890</v>
       </c>
       <c r="I1258" t="n">
         <v>1728</v>
@@ -34615,7 +34615,7 @@
         </is>
       </c>
       <c r="H1261" t="n">
-        <v>0</v>
+        <v>127872</v>
       </c>
       <c r="I1261" t="n">
         <v>1728</v>
@@ -34642,7 +34642,7 @@
         </is>
       </c>
       <c r="H1262" t="n">
-        <v>0</v>
+        <v>10368</v>
       </c>
       <c r="I1262" t="n">
         <v>1728</v>
@@ -34669,7 +34669,7 @@
         </is>
       </c>
       <c r="H1263" t="n">
-        <v>0</v>
+        <v>15552</v>
       </c>
       <c r="I1263" t="n">
         <v>1728</v>
@@ -34696,7 +34696,7 @@
         </is>
       </c>
       <c r="H1264" t="n">
-        <v>0</v>
+        <v>3456</v>
       </c>
       <c r="I1264" t="n">
         <v>1728</v>
@@ -34750,7 +34750,7 @@
         </is>
       </c>
       <c r="H1266" t="n">
-        <v>0</v>
+        <v>3051</v>
       </c>
       <c r="I1266" t="n">
         <v>1728</v>
@@ -34777,7 +34777,7 @@
         </is>
       </c>
       <c r="H1267" t="n">
-        <v>0</v>
+        <v>1755</v>
       </c>
       <c r="I1267" t="n">
         <v>1728</v>
@@ -34804,7 +34804,7 @@
         </is>
       </c>
       <c r="H1268" t="n">
-        <v>0</v>
+        <v>3456</v>
       </c>
       <c r="I1268" t="n">
         <v>1728</v>
@@ -34831,7 +34831,7 @@
         </is>
       </c>
       <c r="H1269" t="n">
-        <v>0</v>
+        <v>1782</v>
       </c>
       <c r="I1269" t="n">
         <v>1728</v>
@@ -34858,7 +34858,7 @@
         </is>
       </c>
       <c r="H1270" t="n">
-        <v>0</v>
+        <v>5616</v>
       </c>
       <c r="I1270" t="n">
         <v>1728</v>
@@ -34885,7 +34885,7 @@
         </is>
       </c>
       <c r="H1271" t="n">
-        <v>0</v>
+        <v>15552</v>
       </c>
       <c r="I1271" t="n">
         <v>1728</v>
@@ -34912,7 +34912,7 @@
         </is>
       </c>
       <c r="H1272" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I1272" t="n">
         <v>1728</v>
@@ -35182,7 +35182,7 @@
         </is>
       </c>
       <c r="H1282" t="n">
-        <v>0</v>
+        <v>19425</v>
       </c>
       <c r="I1282" t="n">
         <v>1728</v>
@@ -35371,7 +35371,7 @@
         </is>
       </c>
       <c r="H1289" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I1289" t="n">
         <v>1728</v>
@@ -35398,7 +35398,7 @@
         </is>
       </c>
       <c r="H1290" t="n">
-        <v>0</v>
+        <v>41580</v>
       </c>
       <c r="I1290" t="n">
         <v>1728</v>
@@ -35425,7 +35425,7 @@
         </is>
       </c>
       <c r="H1291" t="n">
-        <v>0</v>
+        <v>55296</v>
       </c>
       <c r="I1291" t="n">
         <v>1728</v>
@@ -35452,7 +35452,7 @@
         </is>
       </c>
       <c r="H1292" t="n">
-        <v>0</v>
+        <v>36288</v>
       </c>
       <c r="I1292" t="n">
         <v>1728</v>
@@ -35533,7 +35533,7 @@
         </is>
       </c>
       <c r="H1295" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I1295" t="n">
         <v>1728</v>
@@ -35560,7 +35560,7 @@
         </is>
       </c>
       <c r="H1296" t="n">
-        <v>3672</v>
+        <v>0</v>
       </c>
       <c r="I1296" t="n">
         <v>1728</v>
@@ -35614,7 +35614,7 @@
         </is>
       </c>
       <c r="H1298" t="n">
-        <v>0</v>
+        <v>39744</v>
       </c>
       <c r="I1298" t="n">
         <v>1728</v>
@@ -35668,7 +35668,7 @@
         </is>
       </c>
       <c r="H1300" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I1300" t="n">
         <v>1728</v>
@@ -35779,7 +35779,7 @@
         </is>
       </c>
       <c r="H1304" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I1304" t="n">
         <v>1728</v>
@@ -35860,7 +35860,7 @@
         </is>
       </c>
       <c r="H1307" t="n">
-        <v>0</v>
+        <v>17280</v>
       </c>
       <c r="I1307" t="n">
         <v>1728</v>
@@ -35887,7 +35887,7 @@
         </is>
       </c>
       <c r="H1308" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I1308" t="n">
         <v>1728</v>
@@ -35914,7 +35914,7 @@
         </is>
       </c>
       <c r="H1309" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I1309" t="n">
         <v>1728</v>
@@ -35941,7 +35941,7 @@
         </is>
       </c>
       <c r="H1310" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I1310" t="n">
         <v>1728</v>
@@ -35968,7 +35968,7 @@
         </is>
       </c>
       <c r="H1311" t="n">
-        <v>0</v>
+        <v>1728</v>
       </c>
       <c r="I1311" t="n">
         <v>1728</v>
@@ -36157,7 +36157,7 @@
         </is>
       </c>
       <c r="H1318" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1318" t="n">
         <v>27</v>
@@ -36184,7 +36184,7 @@
         </is>
       </c>
       <c r="H1319" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1319" t="n">
         <v>27</v>
@@ -36211,7 +36211,7 @@
         </is>
       </c>
       <c r="H1320" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1320" t="n">
         <v>27</v>
@@ -36238,7 +36238,7 @@
         </is>
       </c>
       <c r="H1321" t="n">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I1321" t="n">
         <v>27</v>
@@ -36278,7 +36278,7 @@
         </is>
       </c>
       <c r="H1323" t="n">
-        <v>0</v>
+        <v>864</v>
       </c>
       <c r="I1323" t="n">
         <v>1728</v>
@@ -36291,7 +36291,7 @@
         </is>
       </c>
       <c r="H1324" t="n">
-        <v>0</v>
+        <v>864</v>
       </c>
       <c r="I1324" t="n">
         <v>1728</v>
@@ -36304,7 +36304,7 @@
         </is>
       </c>
       <c r="H1325" t="n">
-        <v>0</v>
+        <v>864</v>
       </c>
       <c r="I1325" t="n">
         <v>1728</v>
@@ -36317,7 +36317,7 @@
         </is>
       </c>
       <c r="H1326" t="n">
-        <v>0</v>
+        <v>864</v>
       </c>
       <c r="I1326" t="n">
         <v>1728</v>
@@ -36330,7 +36330,7 @@
         </is>
       </c>
       <c r="H1327" t="n">
-        <v>0</v>
+        <v>864</v>
       </c>
       <c r="I1327" t="n">
         <v>1728</v>
@@ -36343,7 +36343,7 @@
         </is>
       </c>
       <c r="H1328" t="n">
-        <v>0</v>
+        <v>864</v>
       </c>
       <c r="I1328" t="n">
         <v>1728</v>
@@ -36356,7 +36356,7 @@
         </is>
       </c>
       <c r="H1329" t="n">
-        <v>0</v>
+        <v>864</v>
       </c>
       <c r="I1329" t="n">
         <v>1728</v>
@@ -36369,7 +36369,7 @@
         </is>
       </c>
       <c r="H1330" t="n">
-        <v>0</v>
+        <v>864</v>
       </c>
       <c r="I1330" t="n">
         <v>1728</v>
@@ -36382,7 +36382,7 @@
         </is>
       </c>
       <c r="H1331" t="n">
-        <v>0</v>
+        <v>864</v>
       </c>
       <c r="I1331" t="n">
         <v>1728</v>
@@ -36395,7 +36395,7 @@
         </is>
       </c>
       <c r="H1332" t="n">
-        <v>0</v>
+        <v>864</v>
       </c>
       <c r="I1332" t="n">
         <v>1728</v>
@@ -36408,7 +36408,7 @@
         </is>
       </c>
       <c r="H1333" t="n">
-        <v>0</v>
+        <v>864</v>
       </c>
       <c r="I1333" t="n">
         <v>1728</v>
@@ -36421,7 +36421,7 @@
         </is>
       </c>
       <c r="H1334" t="n">
-        <v>0</v>
+        <v>864</v>
       </c>
       <c r="I1334" t="n">
         <v>1728</v>
@@ -36434,7 +36434,7 @@
         </is>
       </c>
       <c r="H1335" t="n">
-        <v>0</v>
+        <v>864</v>
       </c>
       <c r="I1335" t="n">
         <v>1728</v>
@@ -36447,7 +36447,7 @@
         </is>
       </c>
       <c r="H1336" t="n">
-        <v>0</v>
+        <v>864</v>
       </c>
       <c r="I1336" t="n">
         <v>1728</v>
@@ -36460,7 +36460,7 @@
         </is>
       </c>
       <c r="H1337" t="n">
-        <v>0</v>
+        <v>864</v>
       </c>
       <c r="I1337" t="n">
         <v>1728</v>
@@ -36473,7 +36473,7 @@
         </is>
       </c>
       <c r="H1338" t="n">
-        <v>0</v>
+        <v>864</v>
       </c>
       <c r="I1338" t="n">
         <v>1728</v>
@@ -36486,7 +36486,7 @@
         </is>
       </c>
       <c r="H1339" t="n">
-        <v>0</v>
+        <v>864</v>
       </c>
       <c r="I1339" t="n">
         <v>1728</v>
@@ -36499,7 +36499,7 @@
         </is>
       </c>
       <c r="H1340" t="n">
-        <v>0</v>
+        <v>864</v>
       </c>
       <c r="I1340" t="n">
         <v>1728</v>
@@ -36512,7 +36512,7 @@
         </is>
       </c>
       <c r="H1341" t="n">
-        <v>0</v>
+        <v>864</v>
       </c>
       <c r="I1341" t="n">
         <v>1728</v>

</xml_diff>